<commit_message>
added akita and yamagata
</commit_message>
<xml_diff>
--- a/utils/駅名標.xlsx
+++ b/utils/駅名標.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keisu\my-discord-bot\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC21E81E-D21B-487C-9A39-52416A3AA7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC3172C-EB8D-47EA-A27F-E897D950475C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{D59C1B8B-96E7-492C-A94A-67C6C45EEFA4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="1342">
   <si>
     <t>室蘭本線</t>
     <rPh sb="0" eb="4">
@@ -3447,6 +3447,9 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>陸羽東線</t>
+  </si>
+  <si>
     <t>東新城</t>
   </si>
   <si>
@@ -4116,6 +4119,1065 @@
   <si>
     <t>仙台地下鉄東西線</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>秋田</t>
+  </si>
+  <si>
+    <t>秋田県</t>
+    <rPh sb="2" eb="3">
+      <t>ケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>羽後牛島</t>
+  </si>
+  <si>
+    <t>新屋（秋田）</t>
+  </si>
+  <si>
+    <t>桂根</t>
+  </si>
+  <si>
+    <t>下浜</t>
+  </si>
+  <si>
+    <t>道川</t>
+  </si>
+  <si>
+    <t>岩城みなと</t>
+  </si>
+  <si>
+    <t>羽後亀田</t>
+  </si>
+  <si>
+    <t>折渡</t>
+  </si>
+  <si>
+    <t>羽後岩谷</t>
+  </si>
+  <si>
+    <t>羽後本荘</t>
+  </si>
+  <si>
+    <t>西目</t>
+  </si>
+  <si>
+    <t>仁賀保</t>
+  </si>
+  <si>
+    <t>金浦</t>
+  </si>
+  <si>
+    <t>象潟</t>
+  </si>
+  <si>
+    <t>上浜</t>
+  </si>
+  <si>
+    <t>小砂川</t>
+  </si>
+  <si>
+    <t>羽越本線</t>
+    <rPh sb="0" eb="4">
+      <t>ウエツホンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>羽越本線、奥羽本線、男鹿線、秋田新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>ウエツホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="9">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="10" eb="13">
+      <t>オガセン</t>
+    </rPh>
+    <rPh sb="14" eb="19">
+      <t>アキタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>羽越本線、由利高原鉄道鳥海山ろく線</t>
+    <rPh sb="0" eb="4">
+      <t>ウエツホンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>陣場</t>
+  </si>
+  <si>
+    <t>白沢（秋田）</t>
+  </si>
+  <si>
+    <t>大館</t>
+  </si>
+  <si>
+    <t>下川沿</t>
+  </si>
+  <si>
+    <t>早口</t>
+  </si>
+  <si>
+    <t>糠沢</t>
+  </si>
+  <si>
+    <t>鷹ノ巣</t>
+  </si>
+  <si>
+    <t>前山</t>
+  </si>
+  <si>
+    <t>二ッ井</t>
+  </si>
+  <si>
+    <t>富根</t>
+  </si>
+  <si>
+    <t>鶴形</t>
+  </si>
+  <si>
+    <t>東能代</t>
+  </si>
+  <si>
+    <t>北金岡</t>
+  </si>
+  <si>
+    <t>森岳</t>
+  </si>
+  <si>
+    <t>鹿渡</t>
+  </si>
+  <si>
+    <t>鯉川</t>
+  </si>
+  <si>
+    <t>八郎潟</t>
+  </si>
+  <si>
+    <t>井川さくら</t>
+  </si>
+  <si>
+    <t>羽後飯塚</t>
+  </si>
+  <si>
+    <t>大久保（秋田）</t>
+  </si>
+  <si>
+    <t>追分（秋田）</t>
+  </si>
+  <si>
+    <t>上飯島</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>土崎</t>
+  </si>
+  <si>
+    <t>泉外旭川</t>
+  </si>
+  <si>
+    <t>四ッ小屋</t>
+  </si>
+  <si>
+    <t>和田</t>
+  </si>
+  <si>
+    <t>大張野</t>
+  </si>
+  <si>
+    <t>羽後境</t>
+  </si>
+  <si>
+    <t>峰吉川</t>
+  </si>
+  <si>
+    <t>刈和野</t>
+  </si>
+  <si>
+    <t>神宮寺</t>
+  </si>
+  <si>
+    <t>大曲（秋田）</t>
+  </si>
+  <si>
+    <t>飯詰</t>
+  </si>
+  <si>
+    <t>後三年</t>
+  </si>
+  <si>
+    <t>横手</t>
+  </si>
+  <si>
+    <t>柳田</t>
+  </si>
+  <si>
+    <t>醍醐（秋田）</t>
+  </si>
+  <si>
+    <t>十文字</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>下湯沢</t>
+  </si>
+  <si>
+    <t>湯沢</t>
+  </si>
+  <si>
+    <t>上湯沢</t>
+  </si>
+  <si>
+    <t>三関</t>
+  </si>
+  <si>
+    <t>横堀</t>
+  </si>
+  <si>
+    <t>院内</t>
+  </si>
+  <si>
+    <t>奥羽本線、花輪線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>ハナワセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、五能線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>ゴノウセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、男鹿線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>オガセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、田沢湖線、秋田新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="9">
+      <t>タザワコセン</t>
+    </rPh>
+    <rPh sb="10" eb="15">
+      <t>アキタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、北上線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>キタカミセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>湯瀬温泉</t>
+  </si>
+  <si>
+    <t>八幡平</t>
+  </si>
+  <si>
+    <t>陸中大里</t>
+  </si>
+  <si>
+    <t>鹿角花輪</t>
+  </si>
+  <si>
+    <t>柴平</t>
+  </si>
+  <si>
+    <t>十和田南</t>
+  </si>
+  <si>
+    <t>末広</t>
+  </si>
+  <si>
+    <t>土深井</t>
+  </si>
+  <si>
+    <t>沢尻</t>
+  </si>
+  <si>
+    <t>十二所</t>
+  </si>
+  <si>
+    <t>大滝温泉</t>
+  </si>
+  <si>
+    <t>扇田</t>
+  </si>
+  <si>
+    <t>東大館</t>
+  </si>
+  <si>
+    <t>五能線</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>岩館</t>
+  </si>
+  <si>
+    <t>あきた白神</t>
+  </si>
+  <si>
+    <t>滝ノ間</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>八森</t>
+  </si>
+  <si>
+    <t>東八森</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>沢目</t>
+  </si>
+  <si>
+    <t>鳥形</t>
+  </si>
+  <si>
+    <t>北能代</t>
+  </si>
+  <si>
+    <t>向能代</t>
+  </si>
+  <si>
+    <t>能代</t>
+  </si>
+  <si>
+    <t>出戸浜</t>
+  </si>
+  <si>
+    <t>男鹿線</t>
+    <rPh sb="0" eb="3">
+      <t>オガセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>上二田</t>
+  </si>
+  <si>
+    <t>二田</t>
+  </si>
+  <si>
+    <t>天王</t>
+  </si>
+  <si>
+    <t>船越</t>
+  </si>
+  <si>
+    <t>脇本</t>
+  </si>
+  <si>
+    <t>羽立</t>
+  </si>
+  <si>
+    <t>男鹿</t>
+  </si>
+  <si>
+    <t>田沢湖</t>
+  </si>
+  <si>
+    <t>刺巻</t>
+  </si>
+  <si>
+    <t>神代（秋田）</t>
+  </si>
+  <si>
+    <t>生田（秋田）</t>
+  </si>
+  <si>
+    <t>角館</t>
+  </si>
+  <si>
+    <t>鶯野</t>
+  </si>
+  <si>
+    <t>羽後長野</t>
+  </si>
+  <si>
+    <t>鑓見内</t>
+  </si>
+  <si>
+    <t>羽後四ッ屋</t>
+  </si>
+  <si>
+    <t>北大曲</t>
+  </si>
+  <si>
+    <t>田沢湖線、秋田内陸縦貫鉄道、秋田新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>タザワコセン</t>
+    </rPh>
+    <rPh sb="5" eb="13">
+      <t>アキタナイリクジュウカンテツドウ</t>
+    </rPh>
+    <rPh sb="14" eb="19">
+      <t>アキタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>黒沢（ＪＲ）</t>
+  </si>
+  <si>
+    <t>小松川</t>
+  </si>
+  <si>
+    <t>相野々</t>
+  </si>
+  <si>
+    <t>北上線</t>
+    <rPh sb="0" eb="3">
+      <t>キタカミセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>秋田内陸縦貫鉄道</t>
+  </si>
+  <si>
+    <t>羽後太田</t>
+  </si>
+  <si>
+    <t>西明寺</t>
+  </si>
+  <si>
+    <t>八津</t>
+  </si>
+  <si>
+    <t>羽後長戸呂</t>
+  </si>
+  <si>
+    <t>松葉</t>
+  </si>
+  <si>
+    <t>羽後中里</t>
+  </si>
+  <si>
+    <t>左通</t>
+  </si>
+  <si>
+    <t>上桧木内</t>
+  </si>
+  <si>
+    <t>戸沢</t>
+  </si>
+  <si>
+    <t>阿仁マタギ</t>
+  </si>
+  <si>
+    <t>奥阿仁</t>
+  </si>
+  <si>
+    <t>比立内</t>
+  </si>
+  <si>
+    <t>岩野目</t>
+  </si>
+  <si>
+    <t>笑内</t>
+  </si>
+  <si>
+    <t>萱草</t>
+  </si>
+  <si>
+    <t>荒瀬</t>
+  </si>
+  <si>
+    <t>阿仁合</t>
+  </si>
+  <si>
+    <t>小渕</t>
+  </si>
+  <si>
+    <t>前田南</t>
+  </si>
+  <si>
+    <t>阿仁前田温泉</t>
+  </si>
+  <si>
+    <t>桂瀬</t>
+  </si>
+  <si>
+    <t>米内沢</t>
+  </si>
+  <si>
+    <t>上杉</t>
+  </si>
+  <si>
+    <t>合川</t>
+  </si>
+  <si>
+    <t>大野台</t>
+  </si>
+  <si>
+    <t>縄文小ヶ田</t>
+  </si>
+  <si>
+    <t>西鷹巣</t>
+  </si>
+  <si>
+    <t>鷹巣</t>
+  </si>
+  <si>
+    <t>由利高原鉄道鳥海山ろく線</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>薬師堂（秋田）</t>
+  </si>
+  <si>
+    <t>子吉</t>
+  </si>
+  <si>
+    <t>鮎川（秋田）</t>
+  </si>
+  <si>
+    <t>黒沢（由利高原鉄道）</t>
+  </si>
+  <si>
+    <t>曲沢</t>
+  </si>
+  <si>
+    <t>前郷</t>
+  </si>
+  <si>
+    <t>久保田（秋田）</t>
+  </si>
+  <si>
+    <t>西滝沢</t>
+  </si>
+  <si>
+    <t>吉沢</t>
+  </si>
+  <si>
+    <t>川辺</t>
+  </si>
+  <si>
+    <t>矢島</t>
+  </si>
+  <si>
+    <t>山形県</t>
+    <rPh sb="0" eb="3">
+      <t>ヤマガタケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>女鹿</t>
+  </si>
+  <si>
+    <t>吹浦</t>
+  </si>
+  <si>
+    <t>遊佐</t>
+  </si>
+  <si>
+    <t>南鳥海</t>
+  </si>
+  <si>
+    <t>本楯</t>
+  </si>
+  <si>
+    <t>酒田</t>
+  </si>
+  <si>
+    <t>東酒田</t>
+  </si>
+  <si>
+    <t>砂越</t>
+  </si>
+  <si>
+    <t>北余目</t>
+  </si>
+  <si>
+    <t>余目</t>
+  </si>
+  <si>
+    <t>西袋</t>
+  </si>
+  <si>
+    <t>鶴岡</t>
+  </si>
+  <si>
+    <t>藤島</t>
+    <rPh sb="0" eb="2">
+      <t>フジシマ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>羽前大山</t>
+  </si>
+  <si>
+    <t>羽前水沢</t>
+  </si>
+  <si>
+    <t>三瀬</t>
+  </si>
+  <si>
+    <t>小波渡</t>
+  </si>
+  <si>
+    <t>五十川</t>
+  </si>
+  <si>
+    <t>あつみ温泉</t>
+  </si>
+  <si>
+    <t>小岩川</t>
+  </si>
+  <si>
+    <t>鼠ヶ関</t>
+  </si>
+  <si>
+    <t>板谷</t>
+  </si>
+  <si>
+    <t>峠</t>
+  </si>
+  <si>
+    <t>関根</t>
+  </si>
+  <si>
+    <t>米沢</t>
+  </si>
+  <si>
+    <t>置賜</t>
+  </si>
+  <si>
+    <t>高畠</t>
+  </si>
+  <si>
+    <t>赤湯</t>
+  </si>
+  <si>
+    <t>中川（山形）</t>
+  </si>
+  <si>
+    <t>羽前中山</t>
+  </si>
+  <si>
+    <t>かみのやま温泉</t>
+  </si>
+  <si>
+    <t>茂吉記念館前</t>
+  </si>
+  <si>
+    <t>蔵王</t>
+  </si>
+  <si>
+    <t>山形</t>
+  </si>
+  <si>
+    <t>北山形</t>
+  </si>
+  <si>
+    <t>羽前千歳</t>
+  </si>
+  <si>
+    <t>南出羽</t>
+  </si>
+  <si>
+    <t>漆山（山形）</t>
+  </si>
+  <si>
+    <t>高擶</t>
+  </si>
+  <si>
+    <t>天童南</t>
+  </si>
+  <si>
+    <t>天童</t>
+  </si>
+  <si>
+    <t>乱川</t>
+  </si>
+  <si>
+    <t>神町</t>
+  </si>
+  <si>
+    <t>さくらんぼ東根</t>
+  </si>
+  <si>
+    <t>東根</t>
+  </si>
+  <si>
+    <t>村山（山形）</t>
+  </si>
+  <si>
+    <t>袖崎</t>
+  </si>
+  <si>
+    <t>大石田</t>
+  </si>
+  <si>
+    <t>北大石田</t>
+  </si>
+  <si>
+    <t>芦沢</t>
+  </si>
+  <si>
+    <t>舟形</t>
+  </si>
+  <si>
+    <t>新庄</t>
+  </si>
+  <si>
+    <t>泉田</t>
+  </si>
+  <si>
+    <t>羽前豊里</t>
+  </si>
+  <si>
+    <t>真室川</t>
+  </si>
+  <si>
+    <t>釜淵</t>
+  </si>
+  <si>
+    <t>大滝</t>
+  </si>
+  <si>
+    <t>及位</t>
+  </si>
+  <si>
+    <t>奥羽本線、米坂線、山形新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ヨネサカ</t>
+    </rPh>
+    <rPh sb="7" eb="8">
+      <t>セン</t>
+    </rPh>
+    <rPh sb="9" eb="14">
+      <t>ヤマガタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、山形新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="10">
+      <t>ヤマガタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、山形鉄道フラワー長井線、山形新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="17" eb="22">
+      <t>ヤマガタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、仙山線、左沢線、山形新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>センザンセン</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>アテラザワセン</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ヤマガタ</t>
+    </rPh>
+    <rPh sb="15" eb="18">
+      <t>シンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、仙山線、左沢線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>センザンセン</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>アテラザワセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、仙山線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>センザンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>奥羽本線、陸羽東線、陸羽西線、山形新幹線</t>
+    <rPh sb="0" eb="4">
+      <t>オウウホンセン</t>
+    </rPh>
+    <rPh sb="5" eb="9">
+      <t>リクウヒガシセン</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>リクウ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>ニシ</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>セン</t>
+    </rPh>
+    <rPh sb="15" eb="20">
+      <t>ヤマガタシンカンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>左沢線</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>東金井</t>
+  </si>
+  <si>
+    <t>羽前山辺</t>
+  </si>
+  <si>
+    <t>羽前金沢</t>
+  </si>
+  <si>
+    <t>羽前長崎</t>
+  </si>
+  <si>
+    <t>南寒河江</t>
+  </si>
+  <si>
+    <t>寒河江</t>
+  </si>
+  <si>
+    <t>西寒河江</t>
+  </si>
+  <si>
+    <t>羽前高松</t>
+  </si>
+  <si>
+    <t>柴橋</t>
+  </si>
+  <si>
+    <t>左沢</t>
+  </si>
+  <si>
+    <t>面白山高原</t>
+  </si>
+  <si>
+    <t>山寺</t>
+  </si>
+  <si>
+    <t>高瀬（山形）</t>
+  </si>
+  <si>
+    <t>楯山</t>
+  </si>
+  <si>
+    <t>米坂線</t>
+  </si>
+  <si>
+    <t>南米沢</t>
+  </si>
+  <si>
+    <t>西米沢</t>
+  </si>
+  <si>
+    <t>成島（山形）</t>
+  </si>
+  <si>
+    <t>中郡（山形）</t>
+  </si>
+  <si>
+    <t>羽前小松</t>
+  </si>
+  <si>
+    <t>犬川</t>
+  </si>
+  <si>
+    <t>今泉（山形）</t>
+  </si>
+  <si>
+    <t>萩生</t>
+  </si>
+  <si>
+    <t>羽前椿</t>
+  </si>
+  <si>
+    <t>手ノ子</t>
+  </si>
+  <si>
+    <t>羽前沼沢</t>
+  </si>
+  <si>
+    <t>伊佐領</t>
+  </si>
+  <si>
+    <t>羽前松岡</t>
+  </si>
+  <si>
+    <t>小国</t>
+  </si>
+  <si>
+    <t>米坂線、山形鉄道フラワー長井線</t>
+    <rPh sb="4" eb="8">
+      <t>ヤマガタテツドウ</t>
+    </rPh>
+    <rPh sb="12" eb="15">
+      <t>ナガイセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>陸羽西線</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>升形</t>
+  </si>
+  <si>
+    <t>津谷</t>
+  </si>
+  <si>
+    <t>古口</t>
+  </si>
+  <si>
+    <t>清川</t>
+  </si>
+  <si>
+    <t>狩川</t>
+  </si>
+  <si>
+    <t>南野</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>羽越本線、陸羽西線</t>
+    <rPh sb="0" eb="4">
+      <t>ウエツホンセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>堺田</t>
+  </si>
+  <si>
+    <t>赤倉温泉</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>立小路</t>
+  </si>
+  <si>
+    <t>最上</t>
+  </si>
+  <si>
+    <t>大堀</t>
+  </si>
+  <si>
+    <t>鵜杉</t>
+  </si>
+  <si>
+    <t>瀬見温泉</t>
+  </si>
+  <si>
+    <t>東長沢</t>
+  </si>
+  <si>
+    <t>長沢</t>
+  </si>
+  <si>
+    <t>南新庄</t>
+  </si>
+  <si>
+    <t>南陽市役所</t>
+  </si>
+  <si>
+    <t>宮内（山形）</t>
+  </si>
+  <si>
+    <t>おりはた</t>
+  </si>
+  <si>
+    <t>梨郷</t>
+  </si>
+  <si>
+    <t>西大塚</t>
+  </si>
+  <si>
+    <t>時庭</t>
+  </si>
+  <si>
+    <t>南長井</t>
+  </si>
+  <si>
+    <t>長井</t>
+  </si>
+  <si>
+    <t>あやめ公園</t>
+  </si>
+  <si>
+    <t>羽前成田</t>
+  </si>
+  <si>
+    <t>白兎</t>
+  </si>
+  <si>
+    <t>蚕桑</t>
+  </si>
+  <si>
+    <t>鮎貝</t>
+  </si>
+  <si>
+    <t>四季の郷</t>
+  </si>
+  <si>
+    <t>荒砥</t>
+  </si>
+  <si>
+    <t>山形鉄道フラワー長井線</t>
   </si>
 </sst>
 </file>
@@ -4522,7 +5584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1437605C-2F57-4CF5-BCCA-5114B2B10271}">
-  <dimension ref="A1:B945"/>
+  <dimension ref="A1:B1212"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="64.33203125" customWidth="1"/>
@@ -10586,7 +11648,7 @@
         <v>842</v>
       </c>
       <c r="B765" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
     </row>
     <row r="766" spans="1:2">
@@ -10594,7 +11656,7 @@
         <v>843</v>
       </c>
       <c r="B766" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
     </row>
     <row r="767" spans="1:2">
@@ -10602,7 +11664,7 @@
         <v>844</v>
       </c>
       <c r="B767" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
     </row>
     <row r="768" spans="1:2">
@@ -10610,7 +11672,7 @@
         <v>845</v>
       </c>
       <c r="B768" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
     </row>
     <row r="769" spans="1:2">
@@ -10831,7 +11893,7 @@
     </row>
     <row r="796" spans="1:2">
       <c r="A796" s="2" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B796" t="s">
         <v>853</v>
@@ -10839,527 +11901,527 @@
     </row>
     <row r="797" spans="1:2">
       <c r="A797" s="2" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B797" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
     </row>
     <row r="798" spans="1:2">
       <c r="A798" s="2" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="B798" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
     </row>
     <row r="799" spans="1:2">
       <c r="A799" s="2" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B799" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
     </row>
     <row r="800" spans="1:2">
       <c r="A800" s="2" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B800" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="801" spans="1:2">
       <c r="A801" s="2" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="B801" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="802" spans="1:2">
       <c r="A802" s="2" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B802" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="803" spans="1:2">
       <c r="A803" s="2" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B803" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
     </row>
     <row r="804" spans="1:2">
       <c r="A804" s="2" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="B804" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
     </row>
     <row r="805" spans="1:2">
       <c r="A805" s="2" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B805" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="806" spans="1:2">
       <c r="A806" s="2" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="B806" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="807" spans="1:2">
       <c r="A807" s="2" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B807" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="808" spans="1:2">
       <c r="A808" s="2" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="B808" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="809" spans="1:2">
       <c r="A809" s="2" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B809" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="810" spans="1:2">
       <c r="A810" s="2" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="B810" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="811" spans="1:2">
       <c r="A811" s="2" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B811" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="812" spans="1:2">
       <c r="A812" s="2" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="B812" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="813" spans="1:2">
       <c r="A813" s="2" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B813" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
     </row>
     <row r="814" spans="1:2">
       <c r="A814" s="2" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B814" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="815" spans="1:2">
       <c r="A815" s="2" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B815" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="816" spans="1:2">
       <c r="A816" s="2" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="B816" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="817" spans="1:2">
       <c r="A817" s="2" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B817" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="818" spans="1:2">
       <c r="A818" s="2" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B818" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="819" spans="1:2">
       <c r="A819" s="2" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B819" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="820" spans="1:2">
       <c r="A820" s="2" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="B820" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="821" spans="1:2">
       <c r="A821" s="2" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="B821" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
     </row>
     <row r="822" spans="1:2">
       <c r="A822" s="2" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B822" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="823" spans="1:2">
       <c r="A823" s="2" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B823" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="824" spans="1:2">
       <c r="A824" s="2" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B824" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="825" spans="1:2">
       <c r="A825" s="2" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="B825" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="826" spans="1:2">
       <c r="A826" s="2" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B826" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="827" spans="1:2">
       <c r="A827" s="2" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="B827" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="828" spans="1:2">
       <c r="A828" s="2" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B828" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="829" spans="1:2">
       <c r="A829" s="2" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="B829" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="830" spans="1:2">
       <c r="A830" s="2" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B830" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="831" spans="1:2">
       <c r="A831" s="2" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B831" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="832" spans="1:2">
       <c r="A832" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="B832" t="s">
         <v>921</v>
-      </c>
-      <c r="B832" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="833" spans="1:2">
       <c r="A833" s="2" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B833" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="834" spans="1:2">
       <c r="A834" s="2" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="B834" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="835" spans="1:2">
       <c r="A835" s="2" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B835" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="836" spans="1:2">
       <c r="A836" s="2" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B836" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="837" spans="1:2">
       <c r="A837" s="2" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="B837" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="838" spans="1:2">
       <c r="A838" s="2" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="B838" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="839" spans="1:2">
       <c r="A839" s="2" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B839" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="840" spans="1:2">
       <c r="A840" s="2" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="B840" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="841" spans="1:2">
       <c r="A841" s="2" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="B841" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="842" spans="1:2">
       <c r="A842" s="2" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="B842" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="843" spans="1:2">
       <c r="A843" s="2" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="B843" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="844" spans="1:2">
       <c r="A844" s="2" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="B844" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="845" spans="1:2">
       <c r="A845" s="2" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B845" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="846" spans="1:2">
       <c r="A846" s="2" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="B846" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="847" spans="1:2">
       <c r="A847" s="2" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="B847" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="848" spans="1:2">
       <c r="A848" s="2" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="B848" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="849" spans="1:2">
       <c r="A849" s="2" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B849" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="850" spans="1:2">
       <c r="A850" s="2" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="B850" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="851" spans="1:2">
       <c r="A851" s="2" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B851" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="852" spans="1:2">
       <c r="A852" s="2" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B852" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="853" spans="1:2">
       <c r="A853" s="2" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B853" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="854" spans="1:2">
       <c r="A854" s="2" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="B854" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="855" spans="1:2">
       <c r="A855" s="2" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="B855" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="856" spans="1:2">
       <c r="A856" s="2" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B856" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="857" spans="1:2">
       <c r="A857" s="2" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B857" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
     </row>
     <row r="858" spans="1:2">
       <c r="A858" s="2" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="B858" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="859" spans="1:2">
       <c r="A859" s="2" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B859" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="860" spans="1:2">
       <c r="A860" s="2" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B860" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="861" spans="1:2">
       <c r="A861" s="2" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B861" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="862" spans="1:2">
       <c r="A862" s="2" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B862" t="s">
         <v>708</v>
@@ -11367,7 +12429,7 @@
     </row>
     <row r="863" spans="1:2">
       <c r="A863" s="2" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B863" t="s">
         <v>708</v>
@@ -11375,7 +12437,7 @@
     </row>
     <row r="864" spans="1:2">
       <c r="A864" s="2" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B864" t="s">
         <v>708</v>
@@ -11383,7 +12445,7 @@
     </row>
     <row r="865" spans="1:2">
       <c r="A865" s="2" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B865" t="s">
         <v>708</v>
@@ -11391,7 +12453,7 @@
     </row>
     <row r="866" spans="1:2">
       <c r="A866" s="2" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B866" t="s">
         <v>708</v>
@@ -11399,31 +12461,31 @@
     </row>
     <row r="867" spans="1:2">
       <c r="A867" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B867" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="868" spans="1:2">
       <c r="A868" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B868" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
     </row>
     <row r="869" spans="1:2">
       <c r="A869" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B869" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
     </row>
     <row r="870" spans="1:2">
       <c r="A870" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B870" t="s">
         <v>764</v>
@@ -11431,7 +12493,7 @@
     </row>
     <row r="871" spans="1:2">
       <c r="A871" s="2" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B871" t="s">
         <v>764</v>
@@ -11439,7 +12501,7 @@
     </row>
     <row r="872" spans="1:2">
       <c r="A872" s="2" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B872" t="s">
         <v>764</v>
@@ -11447,7 +12509,7 @@
     </row>
     <row r="873" spans="1:2">
       <c r="A873" s="2" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B873" t="s">
         <v>764</v>
@@ -11455,7 +12517,7 @@
     </row>
     <row r="874" spans="1:2">
       <c r="A874" s="2" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B874" t="s">
         <v>764</v>
@@ -11463,7 +12525,7 @@
     </row>
     <row r="875" spans="1:2">
       <c r="A875" s="2" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="B875" t="s">
         <v>764</v>
@@ -11471,7 +12533,7 @@
     </row>
     <row r="876" spans="1:2">
       <c r="A876" s="2" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B876" t="s">
         <v>764</v>
@@ -11479,7 +12541,7 @@
     </row>
     <row r="877" spans="1:2">
       <c r="A877" s="2" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B877" t="s">
         <v>764</v>
@@ -11487,7 +12549,7 @@
     </row>
     <row r="878" spans="1:2">
       <c r="A878" s="2" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="B878" t="s">
         <v>764</v>
@@ -11495,7 +12557,7 @@
     </row>
     <row r="879" spans="1:2">
       <c r="A879" s="2" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="B879" t="s">
         <v>764</v>
@@ -11503,7 +12565,7 @@
     </row>
     <row r="880" spans="1:2">
       <c r="A880" s="2" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B880" t="s">
         <v>764</v>
@@ -11511,55 +12573,55 @@
     </row>
     <row r="881" spans="1:2">
       <c r="A881" s="2" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B881" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
     </row>
     <row r="882" spans="1:2">
       <c r="A882" s="2" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B882" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
     </row>
     <row r="883" spans="1:2">
       <c r="A883" s="2" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="B883" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
     </row>
     <row r="884" spans="1:2">
       <c r="A884" s="2" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="B884" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
     </row>
     <row r="885" spans="1:2">
       <c r="A885" s="2" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="B885" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
     </row>
     <row r="886" spans="1:2">
       <c r="A886" s="2" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B886" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
     </row>
     <row r="887" spans="1:2">
       <c r="A887" s="2" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="B887" t="s">
         <v>764</v>
@@ -11567,7 +12629,7 @@
     </row>
     <row r="888" spans="1:2">
       <c r="A888" s="2" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="B888" t="s">
         <v>764</v>
@@ -11575,7 +12637,7 @@
     </row>
     <row r="889" spans="1:2">
       <c r="A889" s="2" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B889" t="s">
         <v>764</v>
@@ -11583,7 +12645,7 @@
     </row>
     <row r="890" spans="1:2">
       <c r="A890" s="2" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="B890" t="s">
         <v>764</v>
@@ -11591,7 +12653,7 @@
     </row>
     <row r="891" spans="1:2">
       <c r="A891" s="2" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="B891" t="s">
         <v>764</v>
@@ -11599,7 +12661,7 @@
     </row>
     <row r="892" spans="1:2">
       <c r="A892" s="2" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="B892" t="s">
         <v>764</v>
@@ -11607,426 +12669,2524 @@
     </row>
     <row r="893" spans="1:2">
       <c r="A893" s="2" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="B893" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
     </row>
     <row r="894" spans="1:2">
       <c r="A894" s="2" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="B894" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
     </row>
     <row r="895" spans="1:2">
       <c r="A895" s="2" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="B895" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="896" spans="1:2">
       <c r="A896" s="2" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B896" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="897" spans="1:2">
       <c r="A897" s="3" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="B897" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="898" spans="1:2">
       <c r="A898" s="2" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="B898" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="899" spans="1:2">
       <c r="A899" s="2" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="B899" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="900" spans="1:2">
       <c r="A900" s="2" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="B900" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="901" spans="1:2">
       <c r="A901" s="2" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="B901" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="902" spans="1:2">
       <c r="A902" s="2" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="B902" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="903" spans="1:2">
       <c r="A903" s="2" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B903" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="904" spans="1:2">
       <c r="A904" s="2" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="B904" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="905" spans="1:2">
       <c r="A905" s="2" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B905" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="906" spans="1:2">
       <c r="A906" s="2" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="B906" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="907" spans="1:2">
       <c r="A907" s="2" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B907" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="908" spans="1:2">
       <c r="A908" s="2" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B908" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="909" spans="1:2">
       <c r="A909" s="2" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="B909" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="910" spans="1:2">
       <c r="A910" s="2" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B910" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="911" spans="1:2">
       <c r="A911" s="2" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B911" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="912" spans="1:2">
       <c r="A912" s="2" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B912" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="913" spans="1:2">
       <c r="A913" s="2" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="B913" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="914" spans="1:2">
       <c r="A914" s="2" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B914" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="915" spans="1:2">
       <c r="A915" s="2" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B915" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="916" spans="1:2">
       <c r="A916" s="2" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B916" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="917" spans="1:2">
       <c r="A917" s="2" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B917" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="918" spans="1:2">
       <c r="A918" s="2" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B918" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="919" spans="1:2">
       <c r="A919" s="2" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="B919" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="920" spans="1:2">
       <c r="A920" s="2" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B920" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="921" spans="1:2">
       <c r="A921" s="2" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="B921" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="922" spans="1:2">
       <c r="A922" s="2" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="B922" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="923" spans="1:2">
       <c r="A923" s="2" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B923" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="924" spans="1:2">
       <c r="A924" s="2" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B924" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="925" spans="1:2">
       <c r="A925" s="2" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B925" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="926" spans="1:2">
       <c r="A926" s="2" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B926" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="927" spans="1:2">
       <c r="A927" s="2" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="B927" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="928" spans="1:2">
       <c r="A928" s="2" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="B928" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="929" spans="1:2">
       <c r="A929" s="2" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="B929" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="930" spans="1:2">
       <c r="A930" s="2" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B930" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="931" spans="1:2">
       <c r="A931" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B931" t="s">
         <v>1034</v>
-      </c>
-      <c r="B931" t="s">
-        <v>1033</v>
       </c>
     </row>
     <row r="932" spans="1:2">
       <c r="A932" s="2" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B932" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="933" spans="1:2">
       <c r="A933" s="2" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="B933" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="934" spans="1:2">
       <c r="A934" s="2" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B934" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="935" spans="1:2">
       <c r="A935" s="2" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="B935" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="936" spans="1:2">
       <c r="A936" s="2" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="B936" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="937" spans="1:2">
       <c r="A937" s="2" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B937" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="938" spans="1:2">
       <c r="A938" s="2" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B938" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="939" spans="1:2">
       <c r="A939" s="2" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B939" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="940" spans="1:2">
       <c r="A940" s="2" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="B940" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="941" spans="1:2">
       <c r="A941" s="2" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="B941" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="942" spans="1:2">
       <c r="A942" s="2" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B942" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="943" spans="1:2">
       <c r="A943" s="2" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B943" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="944" spans="1:2">
       <c r="A944" s="2" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B944" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="945" spans="1:2">
       <c r="A945" s="2" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="B945" t="s">
-        <v>1050</v>
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="948" spans="1:2">
+      <c r="A948" s="2" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="949" spans="1:2">
+      <c r="A949" s="2" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B949" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="950" spans="1:2">
+      <c r="A950" s="2" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B950" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="951" spans="1:2">
+      <c r="A951" s="2" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B951" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="952" spans="1:2">
+      <c r="A952" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B952" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="953" spans="1:2">
+      <c r="A953" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B953" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="954" spans="1:2">
+      <c r="A954" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B954" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="955" spans="1:2">
+      <c r="A955" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B955" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="956" spans="1:2">
+      <c r="A956" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B956" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="957" spans="1:2">
+      <c r="A957" s="2" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B957" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="958" spans="1:2">
+      <c r="A958" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B958" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="959" spans="1:2">
+      <c r="A959" s="2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B959" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="960" spans="1:2">
+      <c r="A960" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B960" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="961" spans="1:2">
+      <c r="A961" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B961" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="962" spans="1:2">
+      <c r="A962" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B962" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="963" spans="1:2">
+      <c r="A963" s="2" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B963" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="964" spans="1:2">
+      <c r="A964" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B964" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="965" spans="1:2">
+      <c r="A965" s="2" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B965" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="966" spans="1:2">
+      <c r="A966" s="2" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B966" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="967" spans="1:2">
+      <c r="A967" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B967" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="968" spans="1:2">
+      <c r="A968" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B968" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="969" spans="1:2">
+      <c r="A969" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B969" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="970" spans="1:2">
+      <c r="A970" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B970" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="971" spans="1:2">
+      <c r="A971" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B971" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="972" spans="1:2">
+      <c r="A972" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B972" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="973" spans="1:2">
+      <c r="A973" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B973" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="974" spans="1:2">
+      <c r="A974" s="2" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B974" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="975" spans="1:2">
+      <c r="A975" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B975" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="976" spans="1:2">
+      <c r="A976" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B976" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="977" spans="1:2">
+      <c r="A977" s="2" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B977" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="978" spans="1:2">
+      <c r="A978" s="2" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B978" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="979" spans="1:2">
+      <c r="A979" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B979" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="980" spans="1:2">
+      <c r="A980" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B980" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="981" spans="1:2">
+      <c r="A981" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B981" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="982" spans="1:2">
+      <c r="A982" s="2" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B982" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="983" spans="1:2">
+      <c r="A983" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B983" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="984" spans="1:2">
+      <c r="A984" s="2" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B984" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="985" spans="1:2">
+      <c r="A985" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B985" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="986" spans="1:2">
+      <c r="A986" s="2" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B986" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="987" spans="1:2">
+      <c r="A987" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B987" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="988" spans="1:2">
+      <c r="A988" s="2" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B988" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="989" spans="1:2">
+      <c r="A989" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B989" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="990" spans="1:2">
+      <c r="A990" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B990" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="991" spans="1:2">
+      <c r="A991" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B991" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="992" spans="1:2">
+      <c r="A992" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B992" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="993" spans="1:2">
+      <c r="A993" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B993" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="994" spans="1:2">
+      <c r="A994" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B994" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="995" spans="1:2">
+      <c r="A995" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B995" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="996" spans="1:2">
+      <c r="A996" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B996" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="997" spans="1:2">
+      <c r="A997" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B997" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="998" spans="1:2">
+      <c r="A998" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B998" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="999" spans="1:2">
+      <c r="A999" s="2" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B999" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:2">
+      <c r="A1000" s="2" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B1000" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:2">
+      <c r="A1001" s="2" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B1001" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:2">
+      <c r="A1002" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B1002" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:2">
+      <c r="A1003" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:2">
+      <c r="A1004" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B1004" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:2">
+      <c r="A1005" s="2" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B1005" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:2">
+      <c r="A1006" s="2" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B1006" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:2">
+      <c r="A1007" s="2" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B1007" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:2">
+      <c r="A1008" s="2" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B1008" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:2">
+      <c r="A1009" s="2" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B1009" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:2">
+      <c r="A1010" s="2" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B1010" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:2">
+      <c r="A1011" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B1011" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:2">
+      <c r="A1012" s="2" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B1012" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:2">
+      <c r="A1013" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B1013" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:2">
+      <c r="A1014" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B1014" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:2">
+      <c r="A1015" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B1015" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:2">
+      <c r="A1016" s="2" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B1016" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:2">
+      <c r="A1017" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B1017" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:2">
+      <c r="A1018" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B1018" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:2">
+      <c r="A1019" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B1019" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:2">
+      <c r="A1020" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B1020" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:2">
+      <c r="A1021" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B1021" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:2">
+      <c r="A1022" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B1022" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:2">
+      <c r="A1023" s="2" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B1023" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:2">
+      <c r="A1024" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B1024" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:2">
+      <c r="A1025" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B1025" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:2">
+      <c r="A1026" s="2" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B1026" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:2">
+      <c r="A1027" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B1027" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:2">
+      <c r="A1028" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B1028" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:2">
+      <c r="A1029" s="2" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B1029" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:2">
+      <c r="A1030" s="2" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B1030" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:2">
+      <c r="A1031" s="2" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B1031" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:2">
+      <c r="A1032" s="2" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B1032" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:2">
+      <c r="A1033" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B1033" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:2">
+      <c r="A1034" s="2" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B1034" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:2">
+      <c r="A1035" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B1035" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:2">
+      <c r="A1036" s="2" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B1036" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:2">
+      <c r="A1037" s="2" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B1037" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:2">
+      <c r="A1038" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B1038" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:2">
+      <c r="A1039" s="2" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B1039" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:2">
+      <c r="A1040" s="2" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B1040" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:2">
+      <c r="A1041" s="2" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B1041" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:2">
+      <c r="A1042" s="2" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B1042" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:2">
+      <c r="A1043" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B1043" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:2">
+      <c r="A1044" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B1044" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:2">
+      <c r="A1045" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:2">
+      <c r="A1046" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:2">
+      <c r="A1047" s="2" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B1047" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:2">
+      <c r="A1048" s="2" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B1048" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:2">
+      <c r="A1049" s="2" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B1049" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:2">
+      <c r="A1050" s="2" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B1050" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:2">
+      <c r="A1051" s="2" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B1051" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:2">
+      <c r="A1052" s="2" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B1052" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:2">
+      <c r="A1053" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B1053" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:2">
+      <c r="A1054" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1054" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:2">
+      <c r="A1055" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B1055" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:2">
+      <c r="A1056" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B1056" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:2">
+      <c r="A1057" s="2" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B1057" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:2">
+      <c r="A1058" s="2" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B1058" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:2">
+      <c r="A1059" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B1059" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:2">
+      <c r="A1060" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B1060" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:2">
+      <c r="A1061" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B1061" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:2">
+      <c r="A1062" s="2" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B1062" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:2">
+      <c r="A1063" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B1063" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:2">
+      <c r="A1064" s="2" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B1064" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:2">
+      <c r="A1065" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B1065" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:2">
+      <c r="A1066" s="2" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B1066" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:2">
+      <c r="A1067" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B1067" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:2">
+      <c r="A1068" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B1068" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:2">
+      <c r="A1069" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B1069" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:2">
+      <c r="A1070" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B1070" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:2">
+      <c r="A1071" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B1071" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:2">
+      <c r="A1072" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B1072" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:2">
+      <c r="A1073" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B1073" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:2">
+      <c r="A1074" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B1074" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:2">
+      <c r="A1075" s="2" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B1075" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:2">
+      <c r="A1076" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="B1076" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:2">
+      <c r="A1077" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B1077" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:2">
+      <c r="A1078" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="B1078" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:2">
+      <c r="A1079" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="B1079" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:2">
+      <c r="A1080" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:2">
+      <c r="A1081" s="2" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B1081" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:2">
+      <c r="A1082" s="2" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B1082" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:2">
+      <c r="A1083" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B1083" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:2">
+      <c r="A1084" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B1084" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:2">
+      <c r="A1085" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B1085" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:2">
+      <c r="A1086" s="2" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B1086" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:2">
+      <c r="A1087" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B1087" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:2">
+      <c r="A1088" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B1088" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:2">
+      <c r="A1089" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B1089" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:2">
+      <c r="A1090" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:2">
+      <c r="A1091" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:2">
+      <c r="A1092" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B1092" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:2">
+      <c r="A1095" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:2">
+      <c r="A1096" s="2" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B1096" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:2">
+      <c r="A1097" s="2" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B1097" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:2">
+      <c r="A1098" s="2" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B1098" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:2">
+      <c r="A1099" s="2" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B1099" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:2">
+      <c r="A1100" s="2" t="s">
+        <v>1216</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:2">
+      <c r="A1101" s="2" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B1101" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:2">
+      <c r="A1102" s="2" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B1102" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:2">
+      <c r="A1103" s="2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B1103" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:2">
+      <c r="A1104" s="2" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B1104" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:2">
+      <c r="A1105" s="2" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B1105" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:2">
+      <c r="A1106" s="2" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B1106" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:2">
+      <c r="A1107" s="2" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B1107" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:2">
+      <c r="A1108" s="2" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B1108" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:2">
+      <c r="A1109" s="2" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B1109" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:2">
+      <c r="A1110" s="2" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B1110" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:2">
+      <c r="A1111" s="2" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B1111" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:2">
+      <c r="A1112" s="2" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B1112" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:2">
+      <c r="A1113" s="2" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B1113" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:2">
+      <c r="A1114" s="2" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B1114" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:2">
+      <c r="A1115" s="2" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B1115" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:2">
+      <c r="A1116" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B1116" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:2">
+      <c r="A1117" s="2" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B1117" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:2">
+      <c r="A1118" s="2" t="s">
+        <v>1234</v>
+      </c>
+      <c r="B1118" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:2">
+      <c r="A1119" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B1119" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:2">
+      <c r="A1120" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B1120" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:2">
+      <c r="A1121" s="2" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B1121" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:2">
+      <c r="A1122" s="2" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B1122" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:2">
+      <c r="A1123" s="2" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B1123" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:2">
+      <c r="A1124" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B1124" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:2">
+      <c r="A1125" s="2" t="s">
+        <v>1241</v>
+      </c>
+      <c r="B1125" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:2">
+      <c r="A1126" s="2" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B1126" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:2">
+      <c r="A1127" s="2" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B1127" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:2">
+      <c r="A1128" s="2" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B1128" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:2">
+      <c r="A1129" s="2" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B1129" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:2">
+      <c r="A1130" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B1130" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:2">
+      <c r="A1131" s="2" t="s">
+        <v>1247</v>
+      </c>
+      <c r="B1131" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:2">
+      <c r="A1132" s="2" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B1132" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:2">
+      <c r="A1133" s="2" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B1133" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:2">
+      <c r="A1134" s="2" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B1134" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:2">
+      <c r="A1135" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B1135" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:2">
+      <c r="A1136" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B1136" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:2">
+      <c r="A1137" s="2" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B1137" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:2">
+      <c r="A1138" s="2" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B1138" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:2">
+      <c r="A1139" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="B1139" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:2">
+      <c r="A1140" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B1140" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:2">
+      <c r="A1141" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="B1141" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:2">
+      <c r="A1142" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B1142" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:2">
+      <c r="A1143" s="2" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B1143" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:2">
+      <c r="A1144" s="2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B1144" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:2">
+      <c r="A1145" s="2" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B1145" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:2">
+      <c r="A1146" s="2" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B1146" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:2">
+      <c r="A1147" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="B1147" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:2">
+      <c r="A1148" s="2" t="s">
+        <v>1264</v>
+      </c>
+      <c r="B1148" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:2">
+      <c r="A1149" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B1149" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:2">
+      <c r="A1150" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="B1150" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:2">
+      <c r="A1151" s="2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B1151" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:2">
+      <c r="A1152" s="2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B1152" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:2">
+      <c r="A1153" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B1153" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:2">
+      <c r="A1154" s="2" t="s">
+        <v>1278</v>
+      </c>
+      <c r="B1154" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:2">
+      <c r="A1155" s="2" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B1155" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:2">
+      <c r="A1156" s="2" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B1156" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:2">
+      <c r="A1157" s="2" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B1157" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:2">
+      <c r="A1158" s="2" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B1158" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:2">
+      <c r="A1159" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B1159" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:2">
+      <c r="A1160" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B1160" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:2">
+      <c r="A1161" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B1161" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:2">
+      <c r="A1162" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B1162" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:2">
+      <c r="A1163" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1163" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:2">
+      <c r="A1164" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B1164" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:2">
+      <c r="A1165" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B1165" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:2">
+      <c r="A1166" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B1166" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:2">
+      <c r="A1167" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1167" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:2">
+      <c r="A1168" s="2" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B1168" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:2">
+      <c r="A1169" s="2" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B1169" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:2">
+      <c r="A1170" s="2" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B1170" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:2">
+      <c r="A1171" s="2" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B1171" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:2">
+      <c r="A1172" s="2" t="s">
+        <v>1297</v>
+      </c>
+      <c r="B1172" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:2">
+      <c r="A1173" s="2" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B1173" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:2">
+      <c r="A1174" s="2" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B1174" t="s">
+        <v>1307</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:2">
+      <c r="A1175" s="2" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B1175" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:2">
+      <c r="A1176" s="2" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B1176" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:2">
+      <c r="A1177" s="2" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B1177" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:2">
+      <c r="A1178" s="2" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B1178" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:2">
+      <c r="A1179" s="2" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B1179" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:2">
+      <c r="A1180" s="2" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B1180" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:2">
+      <c r="A1181" s="2" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B1181" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:2">
+      <c r="A1182" s="2" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B1182" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:2">
+      <c r="A1183" s="2" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B1183" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:2">
+      <c r="A1184" s="2" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B1184" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:2">
+      <c r="A1185" s="2" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B1185" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:2">
+      <c r="A1186" s="2" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B1186" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:2">
+      <c r="A1187" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B1187" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:2">
+      <c r="A1188" s="2" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B1188" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:2">
+      <c r="A1189" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B1189" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:2">
+      <c r="A1190" s="2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B1190" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:2">
+      <c r="A1191" s="2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B1191" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:2">
+      <c r="A1192" s="2" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B1192" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:2">
+      <c r="A1193" s="2" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B1193" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:2">
+      <c r="A1194" s="2" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B1194" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:2">
+      <c r="A1195" s="2" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B1195" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:2">
+      <c r="A1196" s="2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B1196" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:2">
+      <c r="A1197" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:2">
+      <c r="A1198" s="2" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:2">
+      <c r="A1199" s="2" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:2">
+      <c r="A1200" s="2" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B1200" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:2">
+      <c r="A1201" s="2" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B1201" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:2">
+      <c r="A1202" s="2" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B1202" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:2">
+      <c r="A1203" s="2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B1203" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:2">
+      <c r="A1204" s="2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="B1204" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:2">
+      <c r="A1205" s="2" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B1205" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:2">
+      <c r="A1206" s="2" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B1206" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:2">
+      <c r="A1207" s="2" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B1207" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:2">
+      <c r="A1208" s="2" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B1208" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:2">
+      <c r="A1209" s="2" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B1209" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:2">
+      <c r="A1210" s="2" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B1210" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:2">
+      <c r="A1211" s="2" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B1211" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:2">
+      <c r="A1212" s="2" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B1212" t="s">
+        <v>1341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>